<commit_message>
Daily log - 2026-09-12
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2218,14 +2218,30 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="14" t="n"/>
-      <c r="H30" s="14" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I30" s="15">
         <f>IF(SUM(B30:F30,H30)=0,"",SUM(B30:F30,H30))</f>
         <v/>
@@ -2234,10 +2250,26 @@
         <f>IF(I30="","",1440-I30)</f>
         <v/>
       </c>
-      <c r="K30" s="16" t="n"/>
-      <c r="L30" s="16" t="n"/>
-      <c r="M30" s="16" t="n"/>
-      <c r="N30" s="17" t="n"/>
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L30" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>I wasted the day.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-13
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2272,14 +2272,30 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>70</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>420</v>
+      </c>
       <c r="I31" s="15">
         <f>IF(SUM(B31:F31,H31)=0,"",SUM(B31:F31,H31))</f>
         <v/>
@@ -2288,10 +2304,26 @@
         <f>IF(I31="","",1440-I31)</f>
         <v/>
       </c>
-      <c r="K31" s="16" t="n"/>
-      <c r="L31" s="16" t="n"/>
-      <c r="M31" s="16" t="n"/>
-      <c r="N31" s="17" t="n"/>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N31" s="17" t="inlineStr">
+        <is>
+          <t>Sunday .</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-14
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2326,14 +2326,30 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="14" t="n"/>
-      <c r="F32" s="14" t="n"/>
-      <c r="G32" s="14" t="n"/>
-      <c r="H32" s="14" t="n"/>
+      <c r="A32" s="23" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>167</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>280</v>
+      </c>
       <c r="I32" s="15">
         <f>IF(SUM(B32:F32,H32)=0,"",SUM(B32:F32,H32))</f>
         <v/>
@@ -2342,10 +2358,26 @@
         <f>IF(I32="","",1440-I32)</f>
         <v/>
       </c>
-      <c r="K32" s="16" t="n"/>
-      <c r="L32" s="16" t="n"/>
-      <c r="M32" s="16" t="n"/>
-      <c r="N32" s="17" t="n"/>
+      <c r="K32" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L32" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>No comments .</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-15
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -151,26 +152,6 @@
       <top style="thin">
         <color rgb="FFB7B7B7"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
       <bottom style="thin">
         <color rgb="FFB7B7B7"/>
       </bottom>
@@ -189,11 +170,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,12 +235,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -518,17 +523,17 @@
   <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="105" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" style="23" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" customHeight="1">
+    <row r="1" ht="22.8" customHeight="1" s="23">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>My Data, My Code</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16.8" customHeight="1">
+    <row r="2" ht="16.8" customHeight="1" s="23">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Daily Activity Tracker — Instructions</t>
@@ -773,83 +778,83 @@
   <dimension ref="A1:N401"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="17.21875" customWidth="1" min="1" max="1"/>
-    <col width="10.77734375" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="4"/>
-    <col width="16.44140625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="17.21875" customWidth="1" style="23" min="1" max="1"/>
+    <col width="10.77734375" customWidth="1" style="23" min="2" max="2"/>
+    <col width="11" customWidth="1" style="23" min="3" max="4"/>
+    <col width="16.44140625" bestFit="1" customWidth="1" style="23" min="5" max="5"/>
+    <col width="11" customWidth="1" style="23" min="6" max="6"/>
+    <col width="13" customWidth="1" style="23" min="7" max="7"/>
+    <col width="14" customWidth="1" style="23" min="8" max="9"/>
+    <col width="15" customWidth="1" style="23" min="10" max="10"/>
+    <col width="13" customWidth="1" style="23" min="11" max="11"/>
+    <col width="15" customWidth="1" style="23" min="12" max="12"/>
+    <col width="12" customWidth="1" style="23" min="13" max="13"/>
+    <col width="28" customWidth="1" style="23" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="23">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>My Data, My Code — Daily Log</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1">
+    <row r="2" ht="19.5" customHeight="1" s="23">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Name:</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>HRITISH RANJAN SAHOO</t>
         </is>
       </c>
       <c r="C2" s="21" t="n"/>
-      <c r="D2" s="22" t="n"/>
+      <c r="D2" s="20" t="n"/>
       <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Registration No.:</t>
         </is>
       </c>
-      <c r="F2" s="20" t="n">
+      <c r="F2" s="19" t="n">
         <v>12603644</v>
       </c>
-      <c r="G2" s="22" t="n"/>
-    </row>
-    <row r="3" ht="19.5" customHeight="1">
+      <c r="G2" s="20" t="n"/>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" s="23">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Course / Section:</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>MCA/D1P2632</t>
         </is>
       </c>
       <c r="C3" s="21" t="n"/>
-      <c r="D3" s="22" t="n"/>
+      <c r="D3" s="20" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Month:</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>AUGUST</t>
         </is>
       </c>
-      <c r="G3" s="22" t="n"/>
+      <c r="G3" s="20" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>All durations in MINUTES. Yellow cells = enter your data. Row 6 is a sample — overwrite it. Rows 2-3: fill your details.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="41.4" customHeight="1">
+    <row r="5" ht="41.4" customHeight="1" s="23">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Date</t>
@@ -921,7 +926,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="57.6" customHeight="1">
+    <row r="6" ht="57.6" customHeight="1" s="23">
       <c r="A6" s="8" t="n">
         <v>46253</v>
       </c>
@@ -975,7 +980,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="43.2" customHeight="1">
+    <row r="7" ht="43.2" customHeight="1" s="23">
       <c r="A7" s="13" t="n">
         <v>46254</v>
       </c>
@@ -1029,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28.8" customHeight="1">
+    <row r="8" ht="28.8" customHeight="1" s="23">
       <c r="A8" s="13" t="n">
         <v>46255</v>
       </c>
@@ -1083,7 +1088,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28.8" customHeight="1">
+    <row r="9" ht="28.8" customHeight="1" s="23">
       <c r="A9" s="13" t="n">
         <v>46256</v>
       </c>
@@ -1191,7 +1196,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28.8" customHeight="1">
+    <row r="11" ht="28.8" customHeight="1" s="23">
       <c r="A11" s="13" t="n">
         <v>46258</v>
       </c>
@@ -1245,7 +1250,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="43.2" customHeight="1">
+    <row r="12" ht="43.2" customHeight="1" s="23">
       <c r="A12" s="13" t="n">
         <v>46259</v>
       </c>
@@ -1353,8 +1358,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28.8" customHeight="1">
-      <c r="A14" s="23" t="n">
+    <row r="14" ht="28.8" customHeight="1" s="23">
+      <c r="A14" s="18" t="n">
         <v>46261</v>
       </c>
       <c r="B14" s="14" t="n">
@@ -1408,7 +1413,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
+      <c r="A15" s="18" t="n">
         <v>46262</v>
       </c>
       <c r="B15" s="14" t="n">
@@ -1457,12 +1462,12 @@
       </c>
       <c r="N15" s="17" t="inlineStr">
         <is>
-          <t>Little bit sad cause today is rakhi but i'm not in my home town.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="n">
+          <t xml:space="preserve">n </t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28.8" customHeight="1" s="23">
+      <c r="A16" s="18" t="n">
         <v>46263</v>
       </c>
       <c r="B16" s="14" t="n">
@@ -1516,7 +1521,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
+      <c r="A17" s="18" t="n">
         <v>46264</v>
       </c>
       <c r="B17" s="14" t="n">
@@ -1570,7 +1575,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
+      <c r="A18" s="18" t="n">
         <v>46265</v>
       </c>
       <c r="B18" s="14" t="n">
@@ -1624,7 +1629,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
+      <c r="A19" s="18" t="n">
         <v>46266</v>
       </c>
       <c r="B19" s="14" t="n">
@@ -1677,8 +1682,8 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="23" t="n">
+    <row r="20" ht="28.8" customHeight="1" s="23">
+      <c r="A20" s="18" t="n">
         <v>46267</v>
       </c>
       <c r="B20" s="14" t="n">
@@ -1731,8 +1736,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="23" t="n">
+    <row r="21" ht="43.2" customHeight="1" s="23">
+      <c r="A21" s="18" t="n">
         <v>46268</v>
       </c>
       <c r="B21" s="14" t="n">
@@ -1786,7 +1791,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
+      <c r="A22" s="18" t="n">
         <v>46269</v>
       </c>
       <c r="B22" s="14" t="n">
@@ -1840,7 +1845,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
+      <c r="A23" s="18" t="n">
         <v>46270</v>
       </c>
       <c r="B23" s="14" t="n">
@@ -1893,8 +1898,8 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="23" t="n">
+    <row r="24" ht="28.8" customHeight="1" s="23">
+      <c r="A24" s="18" t="n">
         <v>46271</v>
       </c>
       <c r="B24" s="14" t="n">
@@ -1948,7 +1953,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
+      <c r="A25" s="18" t="n">
         <v>46272</v>
       </c>
       <c r="B25" s="14" t="n">
@@ -2002,7 +2007,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
+      <c r="A26" s="18" t="n">
         <v>46273</v>
       </c>
       <c r="B26" s="14" t="n">
@@ -2055,8 +2060,8 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="23" t="n">
+    <row r="27" ht="28.8" customHeight="1" s="23">
+      <c r="A27" s="18" t="n">
         <v>46274</v>
       </c>
       <c r="B27" s="14" t="n">
@@ -2110,7 +2115,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
+      <c r="A28" s="18" t="n">
         <v>46275</v>
       </c>
       <c r="B28" s="14" t="n">
@@ -2164,7 +2169,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
+      <c r="A29" s="18" t="n">
         <v>46276</v>
       </c>
       <c r="B29" s="14" t="n">
@@ -2218,7 +2223,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
+      <c r="A30" s="18" t="n">
         <v>46277</v>
       </c>
       <c r="B30" s="14" t="n">
@@ -2272,7 +2277,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
+      <c r="A31" s="18" t="n">
         <v>46278</v>
       </c>
       <c r="B31" s="14" t="n">
@@ -2326,7 +2331,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n">
+      <c r="A32" s="25" t="n">
         <v>46279</v>
       </c>
       <c r="B32" s="14" t="n">
@@ -2380,14 +2385,30 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
+      <c r="A33" s="25" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>200</v>
+      </c>
       <c r="I33" s="15">
         <f>IF(SUM(B33:F33,H33)=0,"",SUM(B33:F33,H33))</f>
         <v/>
@@ -2396,10 +2417,26 @@
         <f>IF(I33="","",1440-I33)</f>
         <v/>
       </c>
-      <c r="K33" s="16" t="n"/>
-      <c r="L33" s="16" t="n"/>
-      <c r="M33" s="16" t="n"/>
-      <c r="N33" s="17" t="n"/>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L33" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t>Unsatisified beacuse i got 58% in CA , just because of lack of efforts which i think i can pu into . I'll be comeback</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-16
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2331,7 +2331,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="n">
+      <c r="A32" s="18" t="n">
         <v>46279</v>
       </c>
       <c r="B32" s="14" t="n">
@@ -2384,7 +2384,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="57.6" customHeight="1" s="23">
       <c r="A33" s="25" t="n">
         <v>46280</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>7</v>
       </c>
       <c r="H33" s="14" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I33" s="15">
         <f>IF(SUM(B33:F33,H33)=0,"",SUM(B33:F33,H33))</f>
@@ -2434,19 +2434,35 @@
       </c>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t>Unsatisified beacuse i got 58% in CA , just because of lack of efforts which i think i can pu into . I'll be comeback</t>
+          <t>Unsatisified beacuse i got 58% in CA , just because of lack of efforts which i think i can put into . I'll be comeback</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n"/>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="14" t="n"/>
-      <c r="H34" s="14" t="n"/>
+      <c r="A34" s="25" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>159</v>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I34" s="15">
         <f>IF(SUM(B34:F34,H34)=0,"",SUM(B34:F34,H34))</f>
         <v/>
@@ -2455,10 +2471,26 @@
         <f>IF(I34="","",1440-I34)</f>
         <v/>
       </c>
-      <c r="K34" s="16" t="n"/>
-      <c r="L34" s="16" t="n"/>
-      <c r="M34" s="16" t="n"/>
-      <c r="N34" s="17" t="n"/>
+      <c r="K34" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L34" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>Nthing such productive.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-17
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2493,14 +2493,30 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n"/>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="14" t="n"/>
-      <c r="G35" s="14" t="n"/>
-      <c r="H35" s="14" t="n"/>
+      <c r="A35" s="25" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B35" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C35" s="14" t="n">
+        <v>139</v>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F35" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>260</v>
+      </c>
       <c r="I35" s="15">
         <f>IF(SUM(B35:F35,H35)=0,"",SUM(B35:F35,H35))</f>
         <v/>
@@ -2509,10 +2525,26 @@
         <f>IF(I35="","",1440-I35)</f>
         <v/>
       </c>
-      <c r="K35" s="16" t="n"/>
-      <c r="L35" s="16" t="n"/>
-      <c r="M35" s="16" t="n"/>
-      <c r="N35" s="17" t="n"/>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L35" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N35" s="17" t="inlineStr">
+        <is>
+          <t>Average Day.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-18
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2547,14 +2547,30 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n"/>
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="14" t="n"/>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="14" t="n"/>
+      <c r="A36" s="25" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>133</v>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>220</v>
+      </c>
       <c r="I36" s="15">
         <f>IF(SUM(B36:F36,H36)=0,"",SUM(B36:F36,H36))</f>
         <v/>
@@ -2563,10 +2579,26 @@
         <f>IF(I36="","",1440-I36)</f>
         <v/>
       </c>
-      <c r="K36" s="16" t="n"/>
-      <c r="L36" s="16" t="n"/>
-      <c r="M36" s="16" t="n"/>
-      <c r="N36" s="17" t="n"/>
+      <c r="K36" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L36" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>Preparing For Analytical CA.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-19
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2601,14 +2601,30 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="14" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
-      <c r="G37" s="14" t="n"/>
-      <c r="H37" s="14" t="n"/>
+      <c r="A37" s="25" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B37" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I37" s="15">
         <f>IF(SUM(B37:F37,H37)=0,"",SUM(B37:F37,H37))</f>
         <v/>
@@ -2617,10 +2633,26 @@
         <f>IF(I37="","",1440-I37)</f>
         <v/>
       </c>
-      <c r="K37" s="16" t="n"/>
-      <c r="L37" s="16" t="n"/>
-      <c r="M37" s="16" t="n"/>
-      <c r="N37" s="17" t="n"/>
+      <c r="K37" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L37" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>I could'nt give my best in CA , My expections are not match to my execution . Unhappy.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-20
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2655,14 +2655,30 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n"/>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
-      <c r="G38" s="14" t="n"/>
-      <c r="H38" s="14" t="n"/>
+      <c r="A38" s="25" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B38" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>97</v>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I38" s="15">
         <f>IF(SUM(B38:F38,H38)=0,"",SUM(B38:F38,H38))</f>
         <v/>
@@ -2671,10 +2687,26 @@
         <f>IF(I38="","",1440-I38)</f>
         <v/>
       </c>
-      <c r="K38" s="16" t="n"/>
-      <c r="L38" s="16" t="n"/>
-      <c r="M38" s="16" t="n"/>
-      <c r="N38" s="17" t="n"/>
+      <c r="K38" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L38" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N38" s="17" t="inlineStr">
+        <is>
+          <t>Sunday So , that i do a bunch of cleaning work.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-21
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2709,14 +2709,30 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n"/>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="14" t="n"/>
+      <c r="A39" s="25" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B39" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>160</v>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I39" s="15">
         <f>IF(SUM(B39:F39,H39)=0,"",SUM(B39:F39,H39))</f>
         <v/>
@@ -2725,10 +2741,26 @@
         <f>IF(I39="","",1440-I39)</f>
         <v/>
       </c>
-      <c r="K39" s="16" t="n"/>
-      <c r="L39" s="16" t="n"/>
-      <c r="M39" s="16" t="n"/>
-      <c r="N39" s="17" t="n"/>
+      <c r="K39" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L39" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>Little Unwell .</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-22
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2763,14 +2763,30 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="n"/>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="14" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
-      <c r="G40" s="14" t="n"/>
-      <c r="H40" s="14" t="n"/>
+      <c r="A40" s="25" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B40" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C40" s="14" t="n">
+        <v>112</v>
+      </c>
+      <c r="D40" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>200</v>
+      </c>
       <c r="I40" s="15">
         <f>IF(SUM(B40:F40,H40)=0,"",SUM(B40:F40,H40))</f>
         <v/>
@@ -2779,10 +2795,26 @@
         <f>IF(I40="","",1440-I40)</f>
         <v/>
       </c>
-      <c r="K40" s="16" t="n"/>
-      <c r="L40" s="16" t="n"/>
-      <c r="M40" s="16" t="n"/>
-      <c r="N40" s="17" t="n"/>
+      <c r="K40" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L40" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N40" s="17" t="inlineStr">
+        <is>
+          <t>I want to learn something new .</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-23
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2817,14 +2817,30 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="n"/>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="14" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="14" t="n"/>
-      <c r="G41" s="14" t="n"/>
-      <c r="H41" s="14" t="n"/>
+      <c r="A41" s="25" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B41" s="14" t="n">
+        <v>460</v>
+      </c>
+      <c r="C41" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="D41" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I41" s="15">
         <f>IF(SUM(B41:F41,H41)=0,"",SUM(B41:F41,H41))</f>
         <v/>
@@ -2833,10 +2849,26 @@
         <f>IF(I41="","",1440-I41)</f>
         <v/>
       </c>
-      <c r="K41" s="16" t="n"/>
-      <c r="L41" s="16" t="n"/>
-      <c r="M41" s="16" t="n"/>
-      <c r="N41" s="17" t="n"/>
+      <c r="K41" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L41" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N41" s="17" t="inlineStr">
+        <is>
+          <t>I'm Working on my first minor project.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-24
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2871,14 +2871,30 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="n"/>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="14" t="n"/>
-      <c r="G42" s="14" t="n"/>
-      <c r="H42" s="14" t="n"/>
+      <c r="A42" s="25" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B42" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C42" s="14" t="n">
+        <v>129</v>
+      </c>
+      <c r="D42" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>220</v>
+      </c>
       <c r="I42" s="15">
         <f>IF(SUM(B42:F42,H42)=0,"",SUM(B42:F42,H42))</f>
         <v/>
@@ -2887,10 +2903,26 @@
         <f>IF(I42="","",1440-I42)</f>
         <v/>
       </c>
-      <c r="K42" s="16" t="n"/>
-      <c r="L42" s="16" t="n"/>
-      <c r="M42" s="16" t="n"/>
-      <c r="N42" s="17" t="n"/>
+      <c r="K42" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L42" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N42" s="17" t="inlineStr">
+        <is>
+          <t>Feeling anxious .</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-25
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2925,14 +2925,30 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="n"/>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="14" t="n"/>
-      <c r="D43" s="14" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="14" t="n"/>
-      <c r="G43" s="14" t="n"/>
-      <c r="H43" s="14" t="n"/>
+      <c r="A43" s="25" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B43" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="D43" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F43" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" s="14" t="n">
+        <v>220</v>
+      </c>
       <c r="I43" s="15">
         <f>IF(SUM(B43:F43,H43)=0,"",SUM(B43:F43,H43))</f>
         <v/>
@@ -2941,10 +2957,26 @@
         <f>IF(I43="","",1440-I43)</f>
         <v/>
       </c>
-      <c r="K43" s="16" t="n"/>
-      <c r="L43" s="16" t="n"/>
-      <c r="M43" s="16" t="n"/>
-      <c r="N43" s="17" t="n"/>
+      <c r="K43" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L43" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N43" s="17" t="inlineStr">
+        <is>
+          <t>Working On Python minor project.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-26
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2385,7 +2385,7 @@
       </c>
     </row>
     <row r="33" ht="57.6" customHeight="1" s="23">
-      <c r="A33" s="25" t="n">
+      <c r="A33" s="18" t="n">
         <v>46280</v>
       </c>
       <c r="B33" s="14" t="n">
@@ -2439,7 +2439,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="25" t="n">
+      <c r="A34" s="18" t="n">
         <v>46281</v>
       </c>
       <c r="B34" s="14" t="n">
@@ -2493,7 +2493,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="25" t="n">
+      <c r="A35" s="18" t="n">
         <v>46282</v>
       </c>
       <c r="B35" s="14" t="n">
@@ -2547,7 +2547,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="25" t="n">
+      <c r="A36" s="18" t="n">
         <v>46283</v>
       </c>
       <c r="B36" s="14" t="n">
@@ -2600,8 +2600,8 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="25" t="n">
+    <row r="37" ht="43.2" customHeight="1" s="23">
+      <c r="A37" s="18" t="n">
         <v>46284</v>
       </c>
       <c r="B37" s="14" t="n">
@@ -2654,8 +2654,8 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="25" t="n">
+    <row r="38" ht="28.8" customHeight="1" s="23">
+      <c r="A38" s="18" t="n">
         <v>46285</v>
       </c>
       <c r="B38" s="14" t="n">
@@ -2709,7 +2709,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="25" t="n">
+      <c r="A39" s="18" t="n">
         <v>46286</v>
       </c>
       <c r="B39" s="14" t="n">
@@ -2763,7 +2763,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="25" t="n">
+      <c r="A40" s="18" t="n">
         <v>46287</v>
       </c>
       <c r="B40" s="14" t="n">
@@ -2816,8 +2816,8 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="25" t="n">
+    <row r="41" ht="28.8" customHeight="1" s="23">
+      <c r="A41" s="18" t="n">
         <v>46288</v>
       </c>
       <c r="B41" s="14" t="n">
@@ -2871,7 +2871,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="n">
+      <c r="A42" s="18" t="n">
         <v>46289</v>
       </c>
       <c r="B42" s="14" t="n">
@@ -2924,7 +2924,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="28.8" customHeight="1" s="23">
       <c r="A43" s="25" t="n">
         <v>46290</v>
       </c>
@@ -2979,14 +2979,30 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="13" t="n"/>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="14" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="14" t="n"/>
-      <c r="G44" s="14" t="n"/>
-      <c r="H44" s="14" t="n"/>
+      <c r="A44" s="25" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B44" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I44" s="15">
         <f>IF(SUM(B44:F44,H44)=0,"",SUM(B44:F44,H44))</f>
         <v/>
@@ -2995,10 +3011,26 @@
         <f>IF(I44="","",1440-I44)</f>
         <v/>
       </c>
-      <c r="K44" s="16" t="n"/>
-      <c r="L44" s="16" t="n"/>
-      <c r="M44" s="16" t="n"/>
-      <c r="N44" s="17" t="n"/>
+      <c r="K44" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N44" s="17" t="inlineStr">
+        <is>
+          <t>There was makeup class for Computer Networks.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-27
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3033,14 +3033,30 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="n"/>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="14" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="14" t="n"/>
-      <c r="H45" s="14" t="n"/>
+      <c r="A45" s="25" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B45" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>93</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F45" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I45" s="15">
         <f>IF(SUM(B45:F45,H45)=0,"",SUM(B45:F45,H45))</f>
         <v/>
@@ -3049,10 +3065,26 @@
         <f>IF(I45="","",1440-I45)</f>
         <v/>
       </c>
-      <c r="K45" s="16" t="n"/>
-      <c r="L45" s="16" t="n"/>
-      <c r="M45" s="16" t="n"/>
-      <c r="N45" s="17" t="n"/>
+      <c r="K45" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L45" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N45" s="17" t="inlineStr">
+        <is>
+          <t>I'm worrying about the fact that without prior truth students were  got into roads and damaged property and doing unprecedented things.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-28
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3087,14 +3087,30 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="n"/>
-      <c r="B46" s="14" t="n"/>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="14" t="n"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="14" t="n"/>
-      <c r="G46" s="14" t="n"/>
-      <c r="H46" s="14" t="n"/>
+      <c r="A46" s="25" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B46" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I46" s="15">
         <f>IF(SUM(B46:F46,H46)=0,"",SUM(B46:F46,H46))</f>
         <v/>
@@ -3103,10 +3119,26 @@
         <f>IF(I46="","",1440-I46)</f>
         <v/>
       </c>
-      <c r="K46" s="16" t="n"/>
-      <c r="L46" s="16" t="n"/>
-      <c r="M46" s="16" t="n"/>
-      <c r="N46" s="17" t="n"/>
+      <c r="K46" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N46" s="17" t="inlineStr">
+        <is>
+          <t>I'm on the way to delhi , cause of this unnessesary situation which has took place in our UNI.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-29
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3141,14 +3141,30 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="n"/>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="14" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="14" t="n"/>
-      <c r="H47" s="14" t="n"/>
+      <c r="A47" s="25" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B47" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C47" s="14" t="n">
+        <v>91</v>
+      </c>
+      <c r="D47" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I47" s="15">
         <f>IF(SUM(B47:F47,H47)=0,"",SUM(B47:F47,H47))</f>
         <v/>
@@ -3157,10 +3173,26 @@
         <f>IF(I47="","",1440-I47)</f>
         <v/>
       </c>
-      <c r="K47" s="16" t="n"/>
-      <c r="L47" s="16" t="n"/>
-      <c r="M47" s="16" t="n"/>
-      <c r="N47" s="17" t="n"/>
+      <c r="K47" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L47" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N47" s="17" t="inlineStr">
+        <is>
+          <t>I'm in my friends place , so chilling and vibing .</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-30
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3195,14 +3195,30 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="n"/>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="14" t="n"/>
-      <c r="E48" s="14" t="n"/>
-      <c r="F48" s="14" t="n"/>
-      <c r="G48" s="14" t="n"/>
-      <c r="H48" s="14" t="n"/>
+      <c r="A48" s="25" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B48" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C48" s="14" t="n">
+        <v>77</v>
+      </c>
+      <c r="D48" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I48" s="15">
         <f>IF(SUM(B48:F48,H48)=0,"",SUM(B48:F48,H48))</f>
         <v/>
@@ -3211,10 +3227,26 @@
         <f>IF(I48="","",1440-I48)</f>
         <v/>
       </c>
-      <c r="K48" s="16" t="n"/>
-      <c r="L48" s="16" t="n"/>
-      <c r="M48" s="16" t="n"/>
-      <c r="N48" s="17" t="n"/>
+      <c r="K48" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L48" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N48" s="17" t="inlineStr">
+        <is>
+          <t>I'm covering some geopoliticals moves .</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-01
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3249,14 +3249,30 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="n"/>
-      <c r="B49" s="14" t="n"/>
-      <c r="C49" s="14" t="n"/>
-      <c r="D49" s="14" t="n"/>
-      <c r="E49" s="14" t="n"/>
-      <c r="F49" s="14" t="n"/>
-      <c r="G49" s="14" t="n"/>
-      <c r="H49" s="14" t="n"/>
+      <c r="A49" s="25" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B49" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C49" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="D49" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F49" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14" t="n">
+        <v>360</v>
+      </c>
       <c r="I49" s="15">
         <f>IF(SUM(B49:F49,H49)=0,"",SUM(B49:F49,H49))</f>
         <v/>
@@ -3265,10 +3281,26 @@
         <f>IF(I49="","",1440-I49)</f>
         <v/>
       </c>
-      <c r="K49" s="16" t="n"/>
-      <c r="L49" s="16" t="n"/>
-      <c r="M49" s="16" t="n"/>
-      <c r="N49" s="17" t="n"/>
+      <c r="K49" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L49" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N49" s="17" t="inlineStr">
+        <is>
+          <t>Its a hectic day.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-02
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3303,14 +3303,30 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="n"/>
-      <c r="B50" s="14" t="n"/>
-      <c r="C50" s="14" t="n"/>
-      <c r="D50" s="14" t="n"/>
-      <c r="E50" s="14" t="n"/>
-      <c r="F50" s="14" t="n"/>
-      <c r="G50" s="14" t="n"/>
-      <c r="H50" s="14" t="n"/>
+      <c r="A50" s="25" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B50" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C50" s="14" t="n">
+        <v>220</v>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14" t="n">
+        <v>500</v>
+      </c>
       <c r="I50" s="15">
         <f>IF(SUM(B50:F50,H50)=0,"",SUM(B50:F50,H50))</f>
         <v/>
@@ -3319,10 +3335,26 @@
         <f>IF(I50="","",1440-I50)</f>
         <v/>
       </c>
-      <c r="K50" s="16" t="n"/>
-      <c r="L50" s="16" t="n"/>
-      <c r="M50" s="16" t="n"/>
-      <c r="N50" s="17" t="n"/>
+      <c r="K50" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L50" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N50" s="17" t="inlineStr">
+        <is>
+          <t>It's one of best day in my life i feel something different roaming around Delhi street's.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-03
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3357,14 +3357,30 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="n"/>
-      <c r="B51" s="14" t="n"/>
-      <c r="C51" s="14" t="n"/>
-      <c r="D51" s="14" t="n"/>
-      <c r="E51" s="14" t="n"/>
-      <c r="F51" s="14" t="n"/>
-      <c r="G51" s="14" t="n"/>
-      <c r="H51" s="14" t="n"/>
+      <c r="A51" s="25" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B51" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C51" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="D51" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="E51" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="F51" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I51" s="15">
         <f>IF(SUM(B51:F51,H51)=0,"",SUM(B51:F51,H51))</f>
         <v/>
@@ -3373,10 +3389,26 @@
         <f>IF(I51="","",1440-I51)</f>
         <v/>
       </c>
-      <c r="K51" s="16" t="n"/>
-      <c r="L51" s="16" t="n"/>
-      <c r="M51" s="16" t="n"/>
-      <c r="N51" s="17" t="n"/>
+      <c r="K51" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L51" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N51" s="17" t="inlineStr">
+        <is>
+          <t>Day 2 at delhi , been to AKSHARDHAM.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-04
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3411,14 +3411,30 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="n"/>
-      <c r="B52" s="14" t="n"/>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="14" t="n"/>
-      <c r="E52" s="14" t="n"/>
-      <c r="F52" s="14" t="n"/>
-      <c r="G52" s="14" t="n"/>
-      <c r="H52" s="14" t="n"/>
+      <c r="A52" s="25" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B52" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C52" s="14" t="n">
+        <v>79</v>
+      </c>
+      <c r="D52" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="14" t="n">
+        <v>360</v>
+      </c>
       <c r="I52" s="15">
         <f>IF(SUM(B52:F52,H52)=0,"",SUM(B52:F52,H52))</f>
         <v/>
@@ -3427,10 +3443,26 @@
         <f>IF(I52="","",1440-I52)</f>
         <v/>
       </c>
-      <c r="K52" s="16" t="n"/>
-      <c r="L52" s="16" t="n"/>
-      <c r="M52" s="16" t="n"/>
-      <c r="N52" s="17" t="n"/>
+      <c r="K52" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L52" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N52" s="17" t="inlineStr">
+        <is>
+          <t>Back to my friends Place in Gurgaon.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-05
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3465,14 +3465,30 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="n"/>
-      <c r="B53" s="14" t="n"/>
-      <c r="C53" s="14" t="n"/>
-      <c r="D53" s="14" t="n"/>
-      <c r="E53" s="14" t="n"/>
-      <c r="F53" s="14" t="n"/>
-      <c r="G53" s="14" t="n"/>
-      <c r="H53" s="14" t="n"/>
+      <c r="A53" s="25" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B53" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C53" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="D53" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E53" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F53" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G53" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I53" s="15">
         <f>IF(SUM(B53:F53,H53)=0,"",SUM(B53:F53,H53))</f>
         <v/>
@@ -3481,10 +3497,26 @@
         <f>IF(I53="","",1440-I53)</f>
         <v/>
       </c>
-      <c r="K53" s="16" t="n"/>
-      <c r="L53" s="16" t="n"/>
-      <c r="M53" s="16" t="n"/>
-      <c r="N53" s="17" t="n"/>
+      <c r="K53" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N53" s="17" t="inlineStr">
+        <is>
+          <t>No comments.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-06
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3519,14 +3519,30 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="n"/>
-      <c r="B54" s="14" t="n"/>
-      <c r="C54" s="14" t="n"/>
-      <c r="D54" s="14" t="n"/>
-      <c r="E54" s="14" t="n"/>
-      <c r="F54" s="14" t="n"/>
-      <c r="G54" s="14" t="n"/>
-      <c r="H54" s="14" t="n"/>
+      <c r="A54" s="25" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B54" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C54" s="14" t="n">
+        <v>86</v>
+      </c>
+      <c r="D54" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F54" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="G54" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H54" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I54" s="15">
         <f>IF(SUM(B54:F54,H54)=0,"",SUM(B54:F54,H54))</f>
         <v/>
@@ -3535,10 +3551,26 @@
         <f>IF(I54="","",1440-I54)</f>
         <v/>
       </c>
-      <c r="K54" s="16" t="n"/>
-      <c r="L54" s="16" t="n"/>
-      <c r="M54" s="16" t="n"/>
-      <c r="N54" s="17" t="n"/>
+      <c r="K54" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L54" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N54" s="17" t="inlineStr">
+        <is>
+          <t>We have our revision claases on online class.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-07
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3573,14 +3573,30 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="n"/>
-      <c r="B55" s="14" t="n"/>
-      <c r="C55" s="14" t="n"/>
-      <c r="D55" s="14" t="n"/>
-      <c r="E55" s="14" t="n"/>
-      <c r="F55" s="14" t="n"/>
-      <c r="G55" s="14" t="n"/>
-      <c r="H55" s="14" t="n"/>
+      <c r="A55" s="25" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B55" s="14" t="n">
+        <v>450</v>
+      </c>
+      <c r="C55" s="14" t="n">
+        <v>92</v>
+      </c>
+      <c r="D55" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E55" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F55" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="G55" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H55" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I55" s="15">
         <f>IF(SUM(B55:F55,H55)=0,"",SUM(B55:F55,H55))</f>
         <v/>
@@ -3589,10 +3605,26 @@
         <f>IF(I55="","",1440-I55)</f>
         <v/>
       </c>
-      <c r="K55" s="16" t="n"/>
-      <c r="L55" s="16" t="n"/>
-      <c r="M55" s="16" t="n"/>
-      <c r="N55" s="17" t="n"/>
+      <c r="K55" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L55" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M55" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N55" s="17" t="inlineStr">
+        <is>
+          <t>I am exploring Gurgaon.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-08
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3627,14 +3627,30 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="n"/>
-      <c r="B56" s="14" t="n"/>
-      <c r="C56" s="14" t="n"/>
-      <c r="D56" s="14" t="n"/>
-      <c r="E56" s="14" t="n"/>
-      <c r="F56" s="14" t="n"/>
-      <c r="G56" s="14" t="n"/>
-      <c r="H56" s="14" t="n"/>
+      <c r="A56" s="25" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B56" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C56" s="14" t="n">
+        <v>76</v>
+      </c>
+      <c r="D56" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E56" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="F56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I56" s="15">
         <f>IF(SUM(B56:F56,H56)=0,"",SUM(B56:F56,H56))</f>
         <v/>
@@ -3643,10 +3659,26 @@
         <f>IF(I56="","",1440-I56)</f>
         <v/>
       </c>
-      <c r="K56" s="16" t="n"/>
-      <c r="L56" s="16" t="n"/>
-      <c r="M56" s="16" t="n"/>
-      <c r="N56" s="17" t="n"/>
+      <c r="K56" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L56" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N56" s="17" t="inlineStr">
+        <is>
+          <t>Exploring some Geopolitical Events happening around the world.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-09
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3681,14 +3681,30 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="n"/>
-      <c r="B57" s="14" t="n"/>
-      <c r="C57" s="14" t="n"/>
-      <c r="D57" s="14" t="n"/>
-      <c r="E57" s="14" t="n"/>
-      <c r="F57" s="14" t="n"/>
-      <c r="G57" s="14" t="n"/>
-      <c r="H57" s="14" t="n"/>
+      <c r="A57" s="25" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B57" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C57" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="D57" s="14" t="n">
+        <v>160</v>
+      </c>
+      <c r="E57" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I57" s="15">
         <f>IF(SUM(B57:F57,H57)=0,"",SUM(B57:F57,H57))</f>
         <v/>
@@ -3697,10 +3713,26 @@
         <f>IF(I57="","",1440-I57)</f>
         <v/>
       </c>
-      <c r="K57" s="16" t="n"/>
-      <c r="L57" s="16" t="n"/>
-      <c r="M57" s="16" t="n"/>
-      <c r="N57" s="17" t="n"/>
+      <c r="K57" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L57" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M57" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N57" s="17" t="inlineStr">
+        <is>
+          <t>Sleepy Day.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-10
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3735,14 +3735,30 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="n"/>
-      <c r="B58" s="14" t="n"/>
-      <c r="C58" s="14" t="n"/>
-      <c r="D58" s="14" t="n"/>
-      <c r="E58" s="14" t="n"/>
-      <c r="F58" s="14" t="n"/>
-      <c r="G58" s="14" t="n"/>
-      <c r="H58" s="14" t="n"/>
+      <c r="A58" s="25" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B58" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C58" s="14" t="n">
+        <v>78</v>
+      </c>
+      <c r="D58" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E58" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="14" t="n">
+        <v>450</v>
+      </c>
       <c r="I58" s="15">
         <f>IF(SUM(B58:F58,H58)=0,"",SUM(B58:F58,H58))</f>
         <v/>
@@ -3751,10 +3767,26 @@
         <f>IF(I58="","",1440-I58)</f>
         <v/>
       </c>
-      <c r="K58" s="16" t="n"/>
-      <c r="L58" s="16" t="n"/>
-      <c r="M58" s="16" t="n"/>
-      <c r="N58" s="17" t="n"/>
+      <c r="K58" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L58" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N58" s="17" t="inlineStr">
+        <is>
+          <t>I feel I'am wasting my talent by not taking actions timely.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-11
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3789,14 +3789,30 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="n"/>
-      <c r="B59" s="14" t="n"/>
-      <c r="C59" s="14" t="n"/>
-      <c r="D59" s="14" t="n"/>
-      <c r="E59" s="14" t="n"/>
-      <c r="F59" s="14" t="n"/>
-      <c r="G59" s="14" t="n"/>
-      <c r="H59" s="14" t="n"/>
+      <c r="A59" s="25" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B59" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C59" s="14" t="n">
+        <v>88</v>
+      </c>
+      <c r="D59" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E59" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F59" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I59" s="15">
         <f>IF(SUM(B59:F59,H59)=0,"",SUM(B59:F59,H59))</f>
         <v/>
@@ -3805,10 +3821,26 @@
         <f>IF(I59="","",1440-I59)</f>
         <v/>
       </c>
-      <c r="K59" s="16" t="n"/>
-      <c r="L59" s="16" t="n"/>
-      <c r="M59" s="16" t="n"/>
-      <c r="N59" s="17" t="n"/>
+      <c r="K59" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L59" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N59" s="17" t="inlineStr">
+        <is>
+          <t>It was sunny sunday.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-12
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3843,14 +3843,30 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="n"/>
-      <c r="B60" s="14" t="n"/>
-      <c r="C60" s="14" t="n"/>
-      <c r="D60" s="14" t="n"/>
-      <c r="E60" s="14" t="n"/>
-      <c r="F60" s="14" t="n"/>
-      <c r="G60" s="14" t="n"/>
-      <c r="H60" s="14" t="n"/>
+      <c r="A60" s="25" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B60" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C60" s="14" t="n">
+        <v>105</v>
+      </c>
+      <c r="D60" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="E60" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F60" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="14" t="n">
+        <v>450</v>
+      </c>
       <c r="I60" s="15">
         <f>IF(SUM(B60:F60,H60)=0,"",SUM(B60:F60,H60))</f>
         <v/>
@@ -3859,10 +3875,26 @@
         <f>IF(I60="","",1440-I60)</f>
         <v/>
       </c>
-      <c r="K60" s="16" t="n"/>
-      <c r="L60" s="16" t="n"/>
-      <c r="M60" s="16" t="n"/>
-      <c r="N60" s="17" t="n"/>
+      <c r="K60" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L60" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N60" s="17" t="inlineStr">
+        <is>
+          <t>Today is First MTT Computer Networks.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-13
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3897,14 +3897,30 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="n"/>
-      <c r="B61" s="14" t="n"/>
-      <c r="C61" s="14" t="n"/>
-      <c r="D61" s="14" t="n"/>
-      <c r="E61" s="14" t="n"/>
-      <c r="F61" s="14" t="n"/>
-      <c r="G61" s="14" t="n"/>
-      <c r="H61" s="14" t="n"/>
+      <c r="A61" s="25" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B61" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="C61" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="D61" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="E61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="14" t="n">
+        <v>450</v>
+      </c>
       <c r="I61" s="15">
         <f>IF(SUM(B61:F61,H61)=0,"",SUM(B61:F61,H61))</f>
         <v/>
@@ -3913,10 +3929,26 @@
         <f>IF(I61="","",1440-I61)</f>
         <v/>
       </c>
-      <c r="K61" s="16" t="n"/>
-      <c r="L61" s="16" t="n"/>
-      <c r="M61" s="16" t="n"/>
-      <c r="N61" s="17" t="n"/>
+      <c r="K61" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L61" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M61" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N61" s="17" t="inlineStr">
+        <is>
+          <t>I couldntn given myself 100% in today's exam .</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-14
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -3951,14 +3951,30 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="n"/>
-      <c r="B62" s="14" t="n"/>
-      <c r="C62" s="14" t="n"/>
-      <c r="D62" s="14" t="n"/>
-      <c r="E62" s="14" t="n"/>
-      <c r="F62" s="14" t="n"/>
-      <c r="G62" s="14" t="n"/>
-      <c r="H62" s="14" t="n"/>
+      <c r="A62" s="25" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B62" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="C62" s="14" t="n">
+        <v>96</v>
+      </c>
+      <c r="D62" s="14" t="n">
+        <v>260</v>
+      </c>
+      <c r="E62" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F62" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I62" s="15">
         <f>IF(SUM(B62:F62,H62)=0,"",SUM(B62:F62,H62))</f>
         <v/>
@@ -3967,10 +3983,26 @@
         <f>IF(I62="","",1440-I62)</f>
         <v/>
       </c>
-      <c r="K62" s="16" t="n"/>
-      <c r="L62" s="16" t="n"/>
-      <c r="M62" s="16" t="n"/>
-      <c r="N62" s="17" t="n"/>
+      <c r="K62" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L62" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N62" s="17" t="inlineStr">
+        <is>
+          <t>I feel some sort of satisfaction after the exam.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-15
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4005,14 +4005,30 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="n"/>
-      <c r="B63" s="14" t="n"/>
-      <c r="C63" s="14" t="n"/>
-      <c r="D63" s="14" t="n"/>
-      <c r="E63" s="14" t="n"/>
-      <c r="F63" s="14" t="n"/>
-      <c r="G63" s="14" t="n"/>
-      <c r="H63" s="14" t="n"/>
+      <c r="A63" s="25" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B63" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C63" s="14" t="n">
+        <v>71</v>
+      </c>
+      <c r="D63" s="14" t="n">
+        <v>220</v>
+      </c>
+      <c r="E63" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F63" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I63" s="15">
         <f>IF(SUM(B63:F63,H63)=0,"",SUM(B63:F63,H63))</f>
         <v/>
@@ -4021,10 +4037,26 @@
         <f>IF(I63="","",1440-I63)</f>
         <v/>
       </c>
-      <c r="K63" s="16" t="n"/>
-      <c r="L63" s="16" t="n"/>
-      <c r="M63" s="16" t="n"/>
-      <c r="N63" s="17" t="n"/>
+      <c r="K63" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L63" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N63" s="17" t="inlineStr">
+        <is>
+          <t>Preparing for my Analytical Skills MTT.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-16
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4059,14 +4059,30 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="n"/>
-      <c r="B64" s="14" t="n"/>
-      <c r="C64" s="14" t="n"/>
-      <c r="D64" s="14" t="n"/>
-      <c r="E64" s="14" t="n"/>
-      <c r="F64" s="14" t="n"/>
-      <c r="G64" s="14" t="n"/>
-      <c r="H64" s="14" t="n"/>
+      <c r="A64" s="25" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B64" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C64" s="14" t="n">
+        <v>92</v>
+      </c>
+      <c r="D64" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="E64" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F64" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I64" s="15">
         <f>IF(SUM(B64:F64,H64)=0,"",SUM(B64:F64,H64))</f>
         <v/>
@@ -4075,10 +4091,26 @@
         <f>IF(I64="","",1440-I64)</f>
         <v/>
       </c>
-      <c r="K64" s="16" t="n"/>
-      <c r="L64" s="16" t="n"/>
-      <c r="M64" s="16" t="n"/>
-      <c r="N64" s="17" t="n"/>
+      <c r="K64" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L64" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N64" s="17" t="inlineStr">
+        <is>
+          <t>Not a good day so far .</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-17
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4113,14 +4113,30 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="n"/>
-      <c r="B65" s="14" t="n"/>
-      <c r="C65" s="14" t="n"/>
-      <c r="D65" s="14" t="n"/>
-      <c r="E65" s="14" t="n"/>
-      <c r="F65" s="14" t="n"/>
-      <c r="G65" s="14" t="n"/>
-      <c r="H65" s="14" t="n"/>
+      <c r="A65" s="25" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B65" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C65" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="D65" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="E65" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F65" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I65" s="15">
         <f>IF(SUM(B65:F65,H65)=0,"",SUM(B65:F65,H65))</f>
         <v/>
@@ -4129,10 +4145,26 @@
         <f>IF(I65="","",1440-I65)</f>
         <v/>
       </c>
-      <c r="K65" s="16" t="n"/>
-      <c r="L65" s="16" t="n"/>
-      <c r="M65" s="16" t="n"/>
-      <c r="N65" s="17" t="n"/>
+      <c r="K65" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L65" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M65" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N65" s="17" t="inlineStr">
+        <is>
+          <t>End Day of MTT.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-18
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4167,14 +4167,30 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="n"/>
-      <c r="B66" s="14" t="n"/>
-      <c r="C66" s="14" t="n"/>
-      <c r="D66" s="14" t="n"/>
-      <c r="E66" s="14" t="n"/>
-      <c r="F66" s="14" t="n"/>
-      <c r="G66" s="14" t="n"/>
-      <c r="H66" s="14" t="n"/>
+      <c r="A66" s="25" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B66" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C66" s="14" t="n">
+        <v>66</v>
+      </c>
+      <c r="D66" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E66" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F66" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I66" s="15">
         <f>IF(SUM(B66:F66,H66)=0,"",SUM(B66:F66,H66))</f>
         <v/>
@@ -4183,10 +4199,26 @@
         <f>IF(I66="","",1440-I66)</f>
         <v/>
       </c>
-      <c r="K66" s="16" t="n"/>
-      <c r="L66" s="16" t="n"/>
-      <c r="M66" s="16" t="n"/>
-      <c r="N66" s="17" t="n"/>
+      <c r="K66" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L66" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N66" s="17" t="inlineStr">
+        <is>
+          <t>It's lazy day Sunday.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-20
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4275,14 +4275,30 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="n"/>
-      <c r="B68" s="14" t="n"/>
-      <c r="C68" s="14" t="n"/>
-      <c r="D68" s="14" t="n"/>
-      <c r="E68" s="14" t="n"/>
-      <c r="F68" s="14" t="n"/>
-      <c r="G68" s="14" t="n"/>
-      <c r="H68" s="14" t="n"/>
+      <c r="A68" s="25" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B68" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C68" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D68" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E68" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="F68" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="14" t="n">
+        <v>400</v>
+      </c>
       <c r="I68" s="15">
         <f>IF(SUM(B68:F68,H68)=0,"",SUM(B68:F68,H68))</f>
         <v/>
@@ -4291,10 +4307,26 @@
         <f>IF(I68="","",1440-I68)</f>
         <v/>
       </c>
-      <c r="K68" s="16" t="n"/>
-      <c r="L68" s="16" t="n"/>
-      <c r="M68" s="16" t="n"/>
-      <c r="N68" s="17" t="n"/>
+      <c r="K68" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L68" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N68" s="17" t="inlineStr">
+        <is>
+          <t>Its Dussehra.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-21
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4329,14 +4329,30 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="n"/>
-      <c r="B69" s="14" t="n"/>
-      <c r="C69" s="14" t="n"/>
-      <c r="D69" s="14" t="n"/>
-      <c r="E69" s="14" t="n"/>
-      <c r="F69" s="14" t="n"/>
-      <c r="G69" s="14" t="n"/>
-      <c r="H69" s="14" t="n"/>
+      <c r="A69" s="25" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B69" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C69" s="14" t="n">
+        <v>105</v>
+      </c>
+      <c r="D69" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E69" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F69" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G69" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H69" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I69" s="15">
         <f>IF(SUM(B69:F69,H69)=0,"",SUM(B69:F69,H69))</f>
         <v/>
@@ -4345,10 +4361,26 @@
         <f>IF(I69="","",1440-I69)</f>
         <v/>
       </c>
-      <c r="K69" s="16" t="n"/>
-      <c r="L69" s="16" t="n"/>
-      <c r="M69" s="16" t="n"/>
-      <c r="N69" s="17" t="n"/>
+      <c r="K69" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L69" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N69" s="17" t="inlineStr">
+        <is>
+          <t>A good day.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-22
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4383,14 +4383,30 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="n"/>
-      <c r="B70" s="14" t="n"/>
-      <c r="C70" s="14" t="n"/>
-      <c r="D70" s="14" t="n"/>
-      <c r="E70" s="14" t="n"/>
-      <c r="F70" s="14" t="n"/>
-      <c r="G70" s="14" t="n"/>
-      <c r="H70" s="14" t="n"/>
+      <c r="A70" s="25" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B70" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C70" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="D70" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E70" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F70" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G70" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H70" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I70" s="15">
         <f>IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
         <v/>
@@ -4399,10 +4415,26 @@
         <f>IF(I70="","",1440-I70)</f>
         <v/>
       </c>
-      <c r="K70" s="16" t="n"/>
-      <c r="L70" s="16" t="n"/>
-      <c r="M70" s="16" t="n"/>
-      <c r="N70" s="17" t="n"/>
+      <c r="K70" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L70" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N70" s="17" t="inlineStr">
+        <is>
+          <t>I am exploring some Pshycological theories.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-23
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4437,14 +4437,30 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="n"/>
-      <c r="B71" s="14" t="n"/>
-      <c r="C71" s="14" t="n"/>
-      <c r="D71" s="14" t="n"/>
-      <c r="E71" s="14" t="n"/>
-      <c r="F71" s="14" t="n"/>
-      <c r="G71" s="14" t="n"/>
-      <c r="H71" s="14" t="n"/>
+      <c r="A71" s="25" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B71" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C71" s="14" t="n">
+        <v>105</v>
+      </c>
+      <c r="D71" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E71" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H71" s="14" t="n">
+        <v>260</v>
+      </c>
       <c r="I71" s="15">
         <f>IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
         <v/>
@@ -4453,10 +4469,26 @@
         <f>IF(I71="","",1440-I71)</f>
         <v/>
       </c>
-      <c r="K71" s="16" t="n"/>
-      <c r="L71" s="16" t="n"/>
-      <c r="M71" s="16" t="n"/>
-      <c r="N71" s="17" t="n"/>
+      <c r="K71" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L71" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N71" s="17" t="inlineStr">
+        <is>
+          <t>Nothing as such.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-24
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4491,14 +4491,30 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="13" t="n"/>
-      <c r="B72" s="14" t="n"/>
-      <c r="C72" s="14" t="n"/>
-      <c r="D72" s="14" t="n"/>
-      <c r="E72" s="14" t="n"/>
-      <c r="F72" s="14" t="n"/>
-      <c r="G72" s="14" t="n"/>
-      <c r="H72" s="14" t="n"/>
+      <c r="A72" s="25" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B72" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="C72" s="14" t="n">
+        <v>660</v>
+      </c>
+      <c r="D72" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="14" t="n">
+        <v>500</v>
+      </c>
       <c r="I72" s="15">
         <f>IF(SUM(B72:F72,H72)=0,"",SUM(B72:F72,H72))</f>
         <v/>
@@ -4507,10 +4523,26 @@
         <f>IF(I72="","",1440-I72)</f>
         <v/>
       </c>
-      <c r="K72" s="16" t="n"/>
-      <c r="L72" s="16" t="n"/>
-      <c r="M72" s="16" t="n"/>
-      <c r="N72" s="17" t="n"/>
+      <c r="K72" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L72" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N72" s="17" t="inlineStr">
+        <is>
+          <t>Fully satisfied and mesmarizing view of Mata Vaisno Devi Katra , enjoying the track and hill to view.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-25
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4545,14 +4545,30 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="n"/>
-      <c r="B73" s="14" t="n"/>
-      <c r="C73" s="14" t="n"/>
-      <c r="D73" s="14" t="n"/>
-      <c r="E73" s="14" t="n"/>
-      <c r="F73" s="14" t="n"/>
-      <c r="G73" s="14" t="n"/>
-      <c r="H73" s="14" t="n"/>
+      <c r="A73" s="25" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B73" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="C73" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D73" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="14" t="n">
+        <v>600</v>
+      </c>
       <c r="I73" s="15">
         <f>IF(SUM(B73:F73,H73)=0,"",SUM(B73:F73,H73))</f>
         <v/>
@@ -4561,10 +4577,26 @@
         <f>IF(I73="","",1440-I73)</f>
         <v/>
       </c>
-      <c r="K73" s="16" t="n"/>
-      <c r="L73" s="16" t="n"/>
-      <c r="M73" s="16" t="n"/>
-      <c r="N73" s="17" t="n"/>
+      <c r="K73" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L73" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N73" s="17" t="inlineStr">
+        <is>
+          <t>Returning to Room after wonderful trip .</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-26
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4599,14 +4599,30 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="n"/>
-      <c r="B74" s="14" t="n"/>
-      <c r="C74" s="14" t="n"/>
-      <c r="D74" s="14" t="n"/>
-      <c r="E74" s="14" t="n"/>
-      <c r="F74" s="14" t="n"/>
-      <c r="G74" s="14" t="n"/>
-      <c r="H74" s="14" t="n"/>
+      <c r="A74" s="25" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B74" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C74" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D74" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E74" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="14" t="n">
+        <v>500</v>
+      </c>
       <c r="I74" s="15">
         <f>IF(SUM(B74:F74,H74)=0,"",SUM(B74:F74,H74))</f>
         <v/>
@@ -4615,10 +4631,26 @@
         <f>IF(I74="","",1440-I74)</f>
         <v/>
       </c>
-      <c r="K74" s="16" t="n"/>
-      <c r="L74" s="16" t="n"/>
-      <c r="M74" s="16" t="n"/>
-      <c r="N74" s="17" t="n"/>
+      <c r="K74" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L74" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M74" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N74" s="17" t="inlineStr">
+        <is>
+          <t>Back to Base .</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-27
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4653,14 +4653,30 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="n"/>
-      <c r="B75" s="14" t="n"/>
-      <c r="C75" s="14" t="n"/>
-      <c r="D75" s="14" t="n"/>
-      <c r="E75" s="14" t="n"/>
-      <c r="F75" s="14" t="n"/>
-      <c r="G75" s="14" t="n"/>
-      <c r="H75" s="14" t="n"/>
+      <c r="A75" s="25" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B75" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C75" s="14" t="n">
+        <v>114</v>
+      </c>
+      <c r="D75" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="E75" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="F75" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G75" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H75" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I75" s="15">
         <f>IF(SUM(B75:F75,H75)=0,"",SUM(B75:F75,H75))</f>
         <v/>
@@ -4669,10 +4685,26 @@
         <f>IF(I75="","",1440-I75)</f>
         <v/>
       </c>
-      <c r="K75" s="16" t="n"/>
-      <c r="L75" s="16" t="n"/>
-      <c r="M75" s="16" t="n"/>
-      <c r="N75" s="17" t="n"/>
+      <c r="K75" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L75" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N75" s="17" t="inlineStr">
+        <is>
+          <t>Classes after a long weekend.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-10-28
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -4707,14 +4707,30 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="13" t="n"/>
-      <c r="B76" s="14" t="n"/>
-      <c r="C76" s="14" t="n"/>
-      <c r="D76" s="14" t="n"/>
-      <c r="E76" s="14" t="n"/>
-      <c r="F76" s="14" t="n"/>
-      <c r="G76" s="14" t="n"/>
-      <c r="H76" s="14" t="n"/>
+      <c r="A76" s="25" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B76" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C76" s="14" t="n">
+        <v>143</v>
+      </c>
+      <c r="D76" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E76" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F76" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="G76" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I76" s="15">
         <f>IF(SUM(B76:F76,H76)=0,"",SUM(B76:F76,H76))</f>
         <v/>
@@ -4723,10 +4739,26 @@
         <f>IF(I76="","",1440-I76)</f>
         <v/>
       </c>
-      <c r="K76" s="16" t="n"/>
-      <c r="L76" s="16" t="n"/>
-      <c r="M76" s="16" t="n"/>
-      <c r="N76" s="17" t="n"/>
+      <c r="K76" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L76" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N76" s="17" t="inlineStr">
+        <is>
+          <t>Did a research on Finance .</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="13" t="n"/>

</xml_diff>